<commit_message>
chore(sistemas): versionar el generador del Excel
El .xlsx estaba commiteado pero el script que lo produce vivía solo en un
directorio temporal de sesión. Cuando Sistemas responda los 3 pendientes,
regenerarlo habría significado rehacerlo a mano sobre el binario.

Queda en scripts/gen-excel-sistemas.py junto a gen-tags.mjs, con ruta de
salida relativa al repo (antes era absoluta a una máquina) y una nota sobre
recalcular el libro después de generarlo: openpyxl escribe las fórmulas del
resumen sin valor cacheado y se verían vacías para quien lo reciba.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
+++ b/public/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Por confirmar" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$62</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$40</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="184">
   <si>
     <t xml:space="preserve">NOVOPAN · Línea 1 — Tags del HMI para el simulador de trazabilidad</t>
   </si>
@@ -528,178 +528,16 @@
     <t xml:space="preserve">NOMBRE INCOMPLETO (ídem). Comment: "Descarga desde silo capa externa kg/h". Mandar crudo en kg/h.</t>
   </si>
   <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WETS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% ⚠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR UNIDAD.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Dens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — densidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — capacidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR UNIDAD: ¿m³ o kg?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_1_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 1 — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Dens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — densidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — capacidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Dens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — densidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — capacidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_D_Bunker_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WETB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — nivel calculado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR UNIDAD: ¿% o m³?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_A1_3_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — peso (900A1.3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_A1_1_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — caudal 1 (900A1.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_A1_2_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — caudal 2 (900A1.2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_B1_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — humedad (902T2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Hum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — humedad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Hum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — humedad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Hum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — humedad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_08_SL7_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — transmisor de nivel (897T4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071_DRY_Hum_out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRYR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Humedad a la salida del secadero</t>
-  </si>
-  <si>
     <t xml:space="preserve">Prensa_metal_detector</t>
   </si>
   <si>
     <t xml:space="preserve">Prensa</t>
   </si>
   <si>
-    <t xml:space="preserve">Metal detectado en el material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendimiento_sec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendimiento del secadero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delta_T_out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Memory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delta T entrada – salida del tambor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">°C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es Memory Real del HMI: puede no existir en el PLC. Si no sale, se omite.</t>
+    <t xml:space="preserve">Metal detectado en el material (detector a 37.69 m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Está en el servidor de Preparación aunque el equipo es de Sección 2.</t>
   </si>
   <si>
     <t xml:space="preserve">Tema</t>
@@ -739,18 +577,6 @@
   </si>
   <si>
     <t xml:space="preserve">Al revés, el simulador marcaría la línea parada justo cuando está corriendo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿El silo que el HMI llama "silo de polvo 8" (nivel_silo8, Access BRNR) alimenta solo al quemador, o también dosifica material a Sección 2?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Producción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En el modelo hay un "Silo 8" que dosifica a Sección 2. Creemos que NO son el mismo.</t>
   </si>
 </sst>
 </file>
@@ -1587,7 +1413,7 @@
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">COUNTA(Tags!C2:C100)</f>
-        <v>61</v>
+        <v>39</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1596,7 +1422,7 @@
       </c>
       <c r="C36" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"1 · Crítico")</f>
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1605,7 +1431,7 @@
       </c>
       <c r="C37" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"2 · Deseado")</f>
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1614,7 +1440,7 @@
       </c>
       <c r="C38" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"3 · Opcional")</f>
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1623,7 +1449,7 @@
       </c>
       <c r="C39" s="13" t="n">
         <f aca="false">COUNTA('Por confirmar'!B2:B40)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1647,7 +1473,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
@@ -2636,7 +2462,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="26" t="s">
         <v>154</v>
       </c>
@@ -2652,556 +2478,18 @@
       <c r="E40" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F40" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="G40" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H40" s="28" t="s">
         <v>170</v>
       </c>
-      <c r="G40" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H40" s="25" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B41" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>172</v>
-      </c>
-      <c r="D41" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E41" s="28" t="s">
-        <v>173</v>
-      </c>
-      <c r="F41" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="G41" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H41" s="28"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B42" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C42" s="27" t="s">
-        <v>174</v>
-      </c>
-      <c r="D42" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E42" s="28" t="s">
-        <v>175</v>
-      </c>
-      <c r="F42" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G42" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H42" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B43" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C43" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="D43" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E43" s="28" t="s">
-        <v>179</v>
-      </c>
-      <c r="F43" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="G43" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H43" s="25"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B44" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C44" s="27" t="s">
-        <v>180</v>
-      </c>
-      <c r="D44" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E44" s="28" t="s">
-        <v>181</v>
-      </c>
-      <c r="F44" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="G44" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H44" s="25"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B45" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C45" s="27" t="s">
-        <v>182</v>
-      </c>
-      <c r="D45" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E45" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="F45" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="G45" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H45" s="28"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B46" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C46" s="27" t="s">
-        <v>184</v>
-      </c>
-      <c r="D46" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E46" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="F46" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G46" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H46" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B47" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C47" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="D47" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E47" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="F47" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="G47" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H47" s="25"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B48" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C48" s="27" t="s">
-        <v>188</v>
-      </c>
-      <c r="D48" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E48" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="F48" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="G48" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H48" s="28"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B49" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C49" s="27" t="s">
-        <v>190</v>
-      </c>
-      <c r="D49" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E49" s="28" t="s">
-        <v>191</v>
-      </c>
-      <c r="F49" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G49" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H49" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B50" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C50" s="27" t="s">
-        <v>192</v>
-      </c>
-      <c r="D50" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E50" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="F50" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G50" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H50" s="25" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B51" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C51" s="27" t="s">
-        <v>196</v>
-      </c>
-      <c r="D51" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E51" s="28" t="s">
-        <v>197</v>
-      </c>
-      <c r="F51" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="G51" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H51" s="28"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B52" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C52" s="27" t="s">
-        <v>198</v>
-      </c>
-      <c r="D52" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E52" s="28" t="s">
-        <v>199</v>
-      </c>
-      <c r="F52" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="G52" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H52" s="28"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B53" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C53" s="27" t="s">
-        <v>200</v>
-      </c>
-      <c r="D53" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E53" s="28" t="s">
-        <v>201</v>
-      </c>
-      <c r="F53" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="G53" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H53" s="28"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B54" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C54" s="27" t="s">
-        <v>202</v>
-      </c>
-      <c r="D54" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E54" s="28" t="s">
-        <v>203</v>
-      </c>
-      <c r="F54" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G54" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H54" s="28"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B55" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C55" s="27" t="s">
-        <v>204</v>
-      </c>
-      <c r="D55" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E55" s="28" t="s">
-        <v>205</v>
-      </c>
-      <c r="F55" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G55" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H55" s="28"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B56" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C56" s="27" t="s">
-        <v>206</v>
-      </c>
-      <c r="D56" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E56" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="F56" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G56" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H56" s="28"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B57" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C57" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="D57" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E57" s="28" t="s">
-        <v>209</v>
-      </c>
-      <c r="F57" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G57" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H57" s="28"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B58" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C58" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="D58" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E58" s="28" t="s">
-        <v>211</v>
-      </c>
-      <c r="F58" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="G58" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H58" s="28"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B59" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C59" s="27" t="s">
-        <v>212</v>
-      </c>
-      <c r="D59" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="E59" s="28" t="s">
-        <v>214</v>
-      </c>
-      <c r="F59" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G59" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H59" s="28"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B60" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C60" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="D60" s="26" t="s">
-        <v>216</v>
-      </c>
-      <c r="E60" s="28" t="s">
-        <v>217</v>
-      </c>
-      <c r="F60" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="G60" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H60" s="28"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B61" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C61" s="27" t="s">
-        <v>218</v>
-      </c>
-      <c r="D61" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="E61" s="28" t="s">
-        <v>219</v>
-      </c>
-      <c r="F61" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G61" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H61" s="28"/>
-    </row>
-    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B62" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C62" s="27" t="s">
-        <v>220</v>
-      </c>
-      <c r="D62" s="26" t="s">
-        <v>221</v>
-      </c>
-      <c r="E62" s="28" t="s">
-        <v>222</v>
-      </c>
-      <c r="F62" s="26" t="s">
-        <v>223</v>
-      </c>
-      <c r="G62" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H62" s="28" t="s">
-        <v>224</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H62"/>
+  <autoFilter ref="A1:H40"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3218,7 +2506,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -3229,30 +2517,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>225</v>
+        <v>171</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>226</v>
+        <v>172</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>227</v>
+        <v>173</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>228</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>229</v>
+        <v>175</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>230</v>
+        <v>176</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>232</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3260,41 +2548,27 @@
         <v>46</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>233</v>
+        <v>179</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>234</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>235</v>
+        <v>181</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>236</v>
+        <v>182</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="30" t="s">
-        <v>238</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>239</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>241</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>